<commit_message>
fdom update and PAR data dump
</commit_message>
<xml_diff>
--- a/Data/aqualog_fdom/SampleDataSheet.xlsx
+++ b/Data/aqualog_fdom/SampleDataSheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Donahue Lab\Desktop\GitHub\biofac\Data\aqualog_fdom\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43E05243-BCE5-4D2B-A50F-932A4DB5DDE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6860A41C-0C60-4D8D-9823-6E9A62353EF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Run1" sheetId="4" r:id="rId1"/>
@@ -18,14 +18,17 @@
     <sheet name="Run3" sheetId="3" r:id="rId3"/>
     <sheet name="Run4" sheetId="6" r:id="rId4"/>
     <sheet name="Run5" sheetId="7" r:id="rId5"/>
-    <sheet name="Blankrun" sheetId="8" r:id="rId6"/>
+    <sheet name="Run6" sheetId="9" r:id="rId6"/>
+    <sheet name="Run7" sheetId="10" r:id="rId7"/>
+    <sheet name="Run8" sheetId="11" r:id="rId8"/>
+    <sheet name="Blankrun" sheetId="8" r:id="rId9"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="487" uniqueCount="428">
   <si>
     <t>SampleNumber</t>
   </si>
@@ -772,16 +775,558 @@
   </si>
   <si>
     <t>BIOFAC_239</t>
+  </si>
+  <si>
+    <t>BIOFAC_240</t>
+  </si>
+  <si>
+    <t>BIOFAC_241</t>
+  </si>
+  <si>
+    <t>BIOFAC_242</t>
+  </si>
+  <si>
+    <t>BIOFAC_243</t>
+  </si>
+  <si>
+    <t>BIOFAC_244</t>
+  </si>
+  <si>
+    <t>BIOFAC_245</t>
+  </si>
+  <si>
+    <t>BIOFAC_246</t>
+  </si>
+  <si>
+    <t>BIOFAC_247</t>
+  </si>
+  <si>
+    <t>BIOFAC_248</t>
+  </si>
+  <si>
+    <t>BIOFAC_249</t>
+  </si>
+  <si>
+    <t>BIOFAC_250</t>
+  </si>
+  <si>
+    <t>BIOFAC_251</t>
+  </si>
+  <si>
+    <t>BIOFAC_252</t>
+  </si>
+  <si>
+    <t>BIOFAC_253</t>
+  </si>
+  <si>
+    <t>BIOFAC_254</t>
+  </si>
+  <si>
+    <t>BIOFAC_255</t>
+  </si>
+  <si>
+    <t>BIOFAC_256</t>
+  </si>
+  <si>
+    <t>BIOFAC_257</t>
+  </si>
+  <si>
+    <t>BIOFAC_258</t>
+  </si>
+  <si>
+    <t>BIOFAC_259</t>
+  </si>
+  <si>
+    <t>BIOFAC_260</t>
+  </si>
+  <si>
+    <t>BIOFAC_261</t>
+  </si>
+  <si>
+    <t>BIOFAC_262</t>
+  </si>
+  <si>
+    <t>BIOFAC_263</t>
+  </si>
+  <si>
+    <t>BIOFAC_264</t>
+  </si>
+  <si>
+    <t>BIOFAC_265</t>
+  </si>
+  <si>
+    <t>BIOFAC_266</t>
+  </si>
+  <si>
+    <t>BIOFAC_267</t>
+  </si>
+  <si>
+    <t>BIOFAC_268</t>
+  </si>
+  <si>
+    <t>BIOFAC_269</t>
+  </si>
+  <si>
+    <t>BIOFAC_270</t>
+  </si>
+  <si>
+    <t>BIOFAC_271</t>
+  </si>
+  <si>
+    <t>BIOFAC_272</t>
+  </si>
+  <si>
+    <t>BIOFAC_273</t>
+  </si>
+  <si>
+    <t>BIOFAC_274</t>
+  </si>
+  <si>
+    <t>BIOFAC_275</t>
+  </si>
+  <si>
+    <t>BIOFAC_276</t>
+  </si>
+  <si>
+    <t>BIOFAC_277</t>
+  </si>
+  <si>
+    <t>BIOFAC_278</t>
+  </si>
+  <si>
+    <t>BIOFAC_279</t>
+  </si>
+  <si>
+    <t>BIOFAC_280</t>
+  </si>
+  <si>
+    <t>BIOFAC_281</t>
+  </si>
+  <si>
+    <t>BIOFAC_282</t>
+  </si>
+  <si>
+    <t>BIOFAC_283</t>
+  </si>
+  <si>
+    <t>BIOFAC_284</t>
+  </si>
+  <si>
+    <t>BIOFAC_285</t>
+  </si>
+  <si>
+    <t>BIOFAC_286</t>
+  </si>
+  <si>
+    <t>BIOFAC_287</t>
+  </si>
+  <si>
+    <t>BIOFAC_288</t>
+  </si>
+  <si>
+    <t>BIOFAC_289</t>
+  </si>
+  <si>
+    <t>BIOFAC_290</t>
+  </si>
+  <si>
+    <t>BIOFAC_291</t>
+  </si>
+  <si>
+    <t>BIOFAC_292</t>
+  </si>
+  <si>
+    <t>BIOFAC_293</t>
+  </si>
+  <si>
+    <t>BIOFAC_294</t>
+  </si>
+  <si>
+    <t>BIOFAC_295</t>
+  </si>
+  <si>
+    <t>BIOFAC_296</t>
+  </si>
+  <si>
+    <t>BIOFAC_297</t>
+  </si>
+  <si>
+    <t>BIOFAC_298</t>
+  </si>
+  <si>
+    <t>BIOFAC_299</t>
+  </si>
+  <si>
+    <t>BIOFAC_300</t>
+  </si>
+  <si>
+    <t>BIOFAC_301</t>
+  </si>
+  <si>
+    <t>BIOFAC_302</t>
+  </si>
+  <si>
+    <t>BIOFAC_303</t>
+  </si>
+  <si>
+    <t>BIOFAC_304</t>
+  </si>
+  <si>
+    <t>BIOFAC_305</t>
+  </si>
+  <si>
+    <t>BIOFAC_306</t>
+  </si>
+  <si>
+    <t>BIOFAC_307</t>
+  </si>
+  <si>
+    <t>BIOFAC_308</t>
+  </si>
+  <si>
+    <t>BIOFAC_309</t>
+  </si>
+  <si>
+    <t>BIOFAC_310</t>
+  </si>
+  <si>
+    <t>BIOFAC_311</t>
+  </si>
+  <si>
+    <t>BIOFAC_312</t>
+  </si>
+  <si>
+    <t>BIOFAC_313</t>
+  </si>
+  <si>
+    <t>BIOFAC_314</t>
+  </si>
+  <si>
+    <t>BIOFAC_315</t>
+  </si>
+  <si>
+    <t>BIOFAC_316</t>
+  </si>
+  <si>
+    <t>BIOFAC_317</t>
+  </si>
+  <si>
+    <t>BIOFAC_318</t>
+  </si>
+  <si>
+    <t>BIOFAC_319</t>
+  </si>
+  <si>
+    <t>BIOFAC_320</t>
+  </si>
+  <si>
+    <t>BIOFAC_321</t>
+  </si>
+  <si>
+    <t>BIOFAC_322</t>
+  </si>
+  <si>
+    <t>BIOFAC_323</t>
+  </si>
+  <si>
+    <t>BIOFAC_324</t>
+  </si>
+  <si>
+    <t>BIOFAC_325</t>
+  </si>
+  <si>
+    <t>BIOFAC_326</t>
+  </si>
+  <si>
+    <t>BIOFAC_327</t>
+  </si>
+  <si>
+    <t>BIOFAC_328</t>
+  </si>
+  <si>
+    <t>BIOFAC_329</t>
+  </si>
+  <si>
+    <t>BIOFAC_330</t>
+  </si>
+  <si>
+    <t>BIOFAC_331</t>
+  </si>
+  <si>
+    <t>BIOFAC_332</t>
+  </si>
+  <si>
+    <t>BIOFAC_333</t>
+  </si>
+  <si>
+    <t>BIOFAC_334</t>
+  </si>
+  <si>
+    <t>BIOFAC_335</t>
+  </si>
+  <si>
+    <t>BIOFAC_336</t>
+  </si>
+  <si>
+    <t>BIOFAC_348</t>
+  </si>
+  <si>
+    <t>BIOFAC_349</t>
+  </si>
+  <si>
+    <t>BIOFAC_350</t>
+  </si>
+  <si>
+    <t>BIOFAC_351</t>
+  </si>
+  <si>
+    <t>BIOFAC_352</t>
+  </si>
+  <si>
+    <t>BIOFAC_353</t>
+  </si>
+  <si>
+    <t>BIOFAC_354</t>
+  </si>
+  <si>
+    <t>BIOFAC_355</t>
+  </si>
+  <si>
+    <t>BIOFAC_356</t>
+  </si>
+  <si>
+    <t>BIOFAC_357</t>
+  </si>
+  <si>
+    <t>BIOFAC_358</t>
+  </si>
+  <si>
+    <t>BIOFAC_359</t>
+  </si>
+  <si>
+    <t>BIOFAC_360</t>
+  </si>
+  <si>
+    <t>BIOFAC_361</t>
+  </si>
+  <si>
+    <t>BIOFAC_362</t>
+  </si>
+  <si>
+    <t>BIOFAC_363</t>
+  </si>
+  <si>
+    <t>BIOFAC_364</t>
+  </si>
+  <si>
+    <t>BIOFAC_365</t>
+  </si>
+  <si>
+    <t>BIOFAC_366</t>
+  </si>
+  <si>
+    <t>BIOFAC_367</t>
+  </si>
+  <si>
+    <t>BIOFAC_368</t>
+  </si>
+  <si>
+    <t>BIOFAC_369</t>
+  </si>
+  <si>
+    <t>BIOFAC_370</t>
+  </si>
+  <si>
+    <t>BIOFAC_371</t>
+  </si>
+  <si>
+    <t>BIOFAC_372</t>
+  </si>
+  <si>
+    <t>BIOFAC_373</t>
+  </si>
+  <si>
+    <t>BIOFAC_374</t>
+  </si>
+  <si>
+    <t>BIOFAC_375</t>
+  </si>
+  <si>
+    <t>BIOFAC_376</t>
+  </si>
+  <si>
+    <t>BIOFAC_377</t>
+  </si>
+  <si>
+    <t>BIOFAC_378</t>
+  </si>
+  <si>
+    <t>BIOFAC_379</t>
+  </si>
+  <si>
+    <t>BIOFAC_380</t>
+  </si>
+  <si>
+    <t>BIOFAC_381</t>
+  </si>
+  <si>
+    <t>BIOFAC_382</t>
+  </si>
+  <si>
+    <t>BIOFAC_383</t>
+  </si>
+  <si>
+    <t>BIOFAC_384</t>
+  </si>
+  <si>
+    <t>BIOFAC_385</t>
+  </si>
+  <si>
+    <t>BIOFAC_386</t>
+  </si>
+  <si>
+    <t>BIOFAC_387</t>
+  </si>
+  <si>
+    <t>BIOFAC_388</t>
+  </si>
+  <si>
+    <t>BIOFAC_389</t>
+  </si>
+  <si>
+    <t>BIOFAC_390</t>
+  </si>
+  <si>
+    <t>BIOFAC_391</t>
+  </si>
+  <si>
+    <t>BIOFAC_392</t>
+  </si>
+  <si>
+    <t>BIOFAC_393</t>
+  </si>
+  <si>
+    <t>BIOFAC_394</t>
+  </si>
+  <si>
+    <t>BIOFAC_395</t>
+  </si>
+  <si>
+    <t>BIOFAC_396</t>
+  </si>
+  <si>
+    <t>BIOFAC_397</t>
+  </si>
+  <si>
+    <t>BIOFAC_398</t>
+  </si>
+  <si>
+    <t>BIOFAC_399</t>
+  </si>
+  <si>
+    <t>BIOFAC_400</t>
+  </si>
+  <si>
+    <t>BIOFAC_401</t>
+  </si>
+  <si>
+    <t>BIOFAC_402</t>
+  </si>
+  <si>
+    <t>BIOFAC_403</t>
+  </si>
+  <si>
+    <t>BIOFAC_404</t>
+  </si>
+  <si>
+    <t>BIOFAC_405</t>
+  </si>
+  <si>
+    <t>BIOFAC_406</t>
+  </si>
+  <si>
+    <t>BIOFAC_407</t>
+  </si>
+  <si>
+    <t>BIOFAC_408</t>
+  </si>
+  <si>
+    <t>BIOFAC_409</t>
+  </si>
+  <si>
+    <t>BIOFAC_410</t>
+  </si>
+  <si>
+    <t>BIOFAC_411</t>
+  </si>
+  <si>
+    <t>BIOFAC_412</t>
+  </si>
+  <si>
+    <t>BIOFAC_413</t>
+  </si>
+  <si>
+    <t>BIOFAC_414</t>
+  </si>
+  <si>
+    <t>BIOFAC_415</t>
+  </si>
+  <si>
+    <t>BIOFAC_416</t>
+  </si>
+  <si>
+    <t>BIOFAC_417</t>
+  </si>
+  <si>
+    <t>BIOFAC_337</t>
+  </si>
+  <si>
+    <t>BIOFAC_338</t>
+  </si>
+  <si>
+    <t>BIOFAC_339</t>
+  </si>
+  <si>
+    <t>BLANK8</t>
+  </si>
+  <si>
+    <t>BIOFAC_340</t>
+  </si>
+  <si>
+    <t>BIOFAC_341</t>
+  </si>
+  <si>
+    <t>BIOFAC_342</t>
+  </si>
+  <si>
+    <t>BIOFAC_343</t>
+  </si>
+  <si>
+    <t>BIOFAC_344</t>
+  </si>
+  <si>
+    <t>BIOFAC_345</t>
+  </si>
+  <si>
+    <t>BIOFAC_346</t>
+  </si>
+  <si>
+    <t>BIOFAC_347</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
@@ -3237,6 +3782,1629 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C2C963C-070C-453A-ABDC-FCBD98D39D11}">
+  <dimension ref="A1:B34"/>
+  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34" t="s">
+        <v>278</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B8F7C16-219F-42CB-8E83-F80250BF1C16}">
+  <dimension ref="A1:B87"/>
+  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>35</v>
+      </c>
+      <c r="B36" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>36</v>
+      </c>
+      <c r="B37" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <v>37</v>
+      </c>
+      <c r="B38" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <v>38</v>
+      </c>
+      <c r="B39" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40">
+        <v>39</v>
+      </c>
+      <c r="B40" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41">
+        <v>40</v>
+      </c>
+      <c r="B41" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42">
+        <v>41</v>
+      </c>
+      <c r="B42" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A43">
+        <v>42</v>
+      </c>
+      <c r="B43" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A44">
+        <v>43</v>
+      </c>
+      <c r="B44" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A45">
+        <v>44</v>
+      </c>
+      <c r="B45" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A46">
+        <v>45</v>
+      </c>
+      <c r="B46" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A47">
+        <v>46</v>
+      </c>
+      <c r="B47" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A48">
+        <v>47</v>
+      </c>
+      <c r="B48" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A49">
+        <v>48</v>
+      </c>
+      <c r="B49" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A50">
+        <v>49</v>
+      </c>
+      <c r="B50" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A51">
+        <v>50</v>
+      </c>
+      <c r="B51" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A52">
+        <v>51</v>
+      </c>
+      <c r="B52" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A53">
+        <v>52</v>
+      </c>
+      <c r="B53" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A54">
+        <v>53</v>
+      </c>
+      <c r="B54" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A55">
+        <v>54</v>
+      </c>
+      <c r="B55" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A56">
+        <v>55</v>
+      </c>
+      <c r="B56" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A57">
+        <v>56</v>
+      </c>
+      <c r="B57" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A58">
+        <v>57</v>
+      </c>
+      <c r="B58" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A59">
+        <v>58</v>
+      </c>
+      <c r="B59" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A60">
+        <v>59</v>
+      </c>
+      <c r="B60" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A61">
+        <v>60</v>
+      </c>
+      <c r="B61" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A62">
+        <v>61</v>
+      </c>
+      <c r="B62" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A63">
+        <v>62</v>
+      </c>
+      <c r="B63" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A64">
+        <v>63</v>
+      </c>
+      <c r="B64" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A65">
+        <v>64</v>
+      </c>
+      <c r="B65" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A66">
+        <v>65</v>
+      </c>
+      <c r="B66" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A67">
+        <v>66</v>
+      </c>
+      <c r="B67" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A68">
+        <v>67</v>
+      </c>
+      <c r="B68" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A69">
+        <v>68</v>
+      </c>
+      <c r="B69" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A70">
+        <v>69</v>
+      </c>
+      <c r="B70" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A71">
+        <v>70</v>
+      </c>
+      <c r="B71" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A72">
+        <v>71</v>
+      </c>
+      <c r="B72" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A73">
+        <v>72</v>
+      </c>
+      <c r="B73" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A74">
+        <v>73</v>
+      </c>
+      <c r="B74" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A75">
+        <v>74</v>
+      </c>
+      <c r="B75" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A76">
+        <v>75</v>
+      </c>
+      <c r="B76" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A77">
+        <v>76</v>
+      </c>
+      <c r="B77" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A78">
+        <v>77</v>
+      </c>
+      <c r="B78" t="s">
+        <v>418</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A79">
+        <v>78</v>
+      </c>
+      <c r="B79" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A80">
+        <v>79</v>
+      </c>
+      <c r="B80" t="s">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A81">
+        <v>80</v>
+      </c>
+      <c r="B81" t="s">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A82">
+        <v>81</v>
+      </c>
+      <c r="B82" t="s">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A83">
+        <v>82</v>
+      </c>
+      <c r="B83" t="s">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A84">
+        <v>83</v>
+      </c>
+      <c r="B84" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A85">
+        <v>84</v>
+      </c>
+      <c r="B85" t="s">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A86">
+        <v>85</v>
+      </c>
+      <c r="B86" t="s">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A87">
+        <v>86</v>
+      </c>
+      <c r="B87" t="s">
+        <v>427</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24F5383B-293F-4DB5-A388-B65AD9E8A28C}">
+  <dimension ref="A1:B78"/>
+  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36">
+        <v>35</v>
+      </c>
+      <c r="B36" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37">
+        <v>36</v>
+      </c>
+      <c r="B37" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38">
+        <v>37</v>
+      </c>
+      <c r="B38" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39">
+        <v>38</v>
+      </c>
+      <c r="B39" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40">
+        <v>39</v>
+      </c>
+      <c r="B40" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41">
+        <v>40</v>
+      </c>
+      <c r="B41" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42">
+        <v>41</v>
+      </c>
+      <c r="B42" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A43">
+        <v>42</v>
+      </c>
+      <c r="B43" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A44">
+        <v>43</v>
+      </c>
+      <c r="B44" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A45">
+        <v>44</v>
+      </c>
+      <c r="B45" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A46">
+        <v>45</v>
+      </c>
+      <c r="B46" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A47">
+        <v>46</v>
+      </c>
+      <c r="B47" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A48">
+        <v>47</v>
+      </c>
+      <c r="B48" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A49">
+        <v>48</v>
+      </c>
+      <c r="B49" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A50">
+        <v>49</v>
+      </c>
+      <c r="B50" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A51">
+        <v>50</v>
+      </c>
+      <c r="B51" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A52">
+        <v>51</v>
+      </c>
+      <c r="B52" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A53">
+        <v>52</v>
+      </c>
+      <c r="B53" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A54">
+        <v>53</v>
+      </c>
+      <c r="B54" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A55">
+        <v>54</v>
+      </c>
+      <c r="B55" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A56">
+        <v>55</v>
+      </c>
+      <c r="B56" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A57">
+        <v>56</v>
+      </c>
+      <c r="B57" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A58">
+        <v>57</v>
+      </c>
+      <c r="B58" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A59">
+        <v>58</v>
+      </c>
+      <c r="B59" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A60">
+        <v>59</v>
+      </c>
+      <c r="B60" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A61">
+        <v>60</v>
+      </c>
+      <c r="B61" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A62">
+        <v>61</v>
+      </c>
+      <c r="B62" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A63">
+        <v>62</v>
+      </c>
+      <c r="B63" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A64">
+        <v>63</v>
+      </c>
+      <c r="B64" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A65">
+        <v>64</v>
+      </c>
+      <c r="B65" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A66">
+        <v>65</v>
+      </c>
+      <c r="B66" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A67">
+        <v>66</v>
+      </c>
+      <c r="B67" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A68">
+        <v>67</v>
+      </c>
+      <c r="B68" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A69">
+        <v>68</v>
+      </c>
+      <c r="B69" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A70">
+        <v>69</v>
+      </c>
+      <c r="B70" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A71">
+        <v>70</v>
+      </c>
+      <c r="B71" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A72">
+        <v>71</v>
+      </c>
+      <c r="B72" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A73">
+        <v>72</v>
+      </c>
+      <c r="B73" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A74">
+        <v>73</v>
+      </c>
+      <c r="B74" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A75">
+        <v>74</v>
+      </c>
+      <c r="B75" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A76">
+        <v>75</v>
+      </c>
+      <c r="B76" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A77">
+        <v>76</v>
+      </c>
+      <c r="B77" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A78">
+        <v>77</v>
+      </c>
+      <c r="B78" t="s">
+        <v>415</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1DF34553-FC16-4C39-B9D7-D6998E16C3C1}">
   <dimension ref="A1:B67"/>
   <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
fDOM processing and outlier analysis
</commit_message>
<xml_diff>
--- a/Data/aqualog_fdom/SampleDataSheet.xlsx
+++ b/Data/aqualog_fdom/SampleDataSheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Donahue Lab\Desktop\GitHub\biofac\Data\aqualog_fdom\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6860A41C-0C60-4D8D-9823-6E9A62353EF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D8574C59-6581-41B3-A4AD-4406D8B2E942}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Run1" sheetId="4" r:id="rId1"/>

</xml_diff>